<commit_message>
AM Pro: Rotalar Siteden Güncellendi
</commit_message>
<xml_diff>
--- a/routes_output.xlsx
+++ b/routes_output.xlsx
@@ -580,28 +580,28 @@
         <v>30</v>
       </c>
       <c r="M2" t="str">
-        <v>1830</v>
+        <v>0</v>
       </c>
       <c r="N2" t="str">
-        <v>346</v>
+        <v>0</v>
       </c>
       <c r="O2" t="str">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="P2" t="str">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="str">
-        <v>$2,768</v>
+        <v>$0</v>
       </c>
       <c r="R2" t="str">
-        <v>$3,682</v>
+        <v>$0</v>
       </c>
       <c r="S2" t="str">
-        <v>$6,366</v>
+        <v>$0</v>
       </c>
       <c r="T2" t="str">
-        <v>$4,795</v>
+        <v>$0</v>
       </c>
       <c r="U2" t="str">
         <v>2191</v>
@@ -723,28 +723,28 @@
         <v>24</v>
       </c>
       <c r="M3" t="str">
-        <v>1396</v>
+        <v>0</v>
       </c>
       <c r="N3" t="str">
-        <v>308</v>
+        <v>0</v>
       </c>
       <c r="O3" t="str">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="P3" t="str">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="str">
-        <v>$2,356</v>
+        <v>$0</v>
       </c>
       <c r="R3" t="str">
-        <v>$3,133</v>
+        <v>$0</v>
       </c>
       <c r="S3" t="str">
-        <v>$5,418</v>
+        <v>$0</v>
       </c>
       <c r="T3" t="str">
-        <v>$4,002</v>
+        <v>$0</v>
       </c>
       <c r="U3" t="str">
         <v>1516</v>
@@ -866,28 +866,28 @@
         <v>27</v>
       </c>
       <c r="M4" t="str">
-        <v>1846</v>
+        <v>0</v>
       </c>
       <c r="N4" t="str">
-        <v>332</v>
+        <v>0</v>
       </c>
       <c r="O4" t="str">
-        <v>104</v>
+        <v>0</v>
       </c>
       <c r="P4" t="str">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="str">
-        <v>$2,735</v>
+        <v>$0</v>
       </c>
       <c r="R4" t="str">
-        <v>$3,637</v>
+        <v>$0</v>
       </c>
       <c r="S4" t="str">
-        <v>$6,289</v>
+        <v>$0</v>
       </c>
       <c r="T4" t="str">
-        <v>$4,736</v>
+        <v>$0</v>
       </c>
       <c r="U4" t="str">
         <v>1945</v>
@@ -1009,28 +1009,28 @@
         <v>25</v>
       </c>
       <c r="M5" t="str">
-        <v>764</v>
+        <v>0</v>
       </c>
       <c r="N5" t="str">
-        <v>244</v>
+        <v>0</v>
       </c>
       <c r="O5" t="str">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="P5" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="str">
-        <v>$2,825</v>
+        <v>$0</v>
       </c>
       <c r="R5" t="str">
-        <v>$3,757</v>
+        <v>$0</v>
       </c>
       <c r="S5" t="str">
-        <v>$6,497</v>
+        <v>$0</v>
       </c>
       <c r="T5" t="str">
-        <v>$4,800</v>
+        <v>$0</v>
       </c>
       <c r="U5" t="str">
         <v>1834</v>
@@ -1295,16 +1295,16 @@
         <v>21</v>
       </c>
       <c r="M7" t="str">
-        <v>1434</v>
+        <v>600</v>
       </c>
       <c r="N7" t="str">
-        <v>254</v>
+        <v>52</v>
       </c>
       <c r="O7" t="str">
-        <v>77</v>
+        <v>16</v>
       </c>
       <c r="P7" t="str">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="str">
         <v>$2,668</v>
@@ -1316,7 +1316,7 @@
         <v>$6,135</v>
       </c>
       <c r="T7" t="str">
-        <v>$4,620</v>
+        <v>$0</v>
       </c>
       <c r="U7" t="str">
         <v>1492</v>
@@ -1581,13 +1581,13 @@
         <v>30</v>
       </c>
       <c r="M9" t="str">
-        <v>912</v>
+        <v>420</v>
       </c>
       <c r="N9" t="str">
-        <v>198</v>
+        <v>72</v>
       </c>
       <c r="O9" t="str">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="P9" t="str">
         <v>0</v>
@@ -2582,16 +2582,16 @@
         <v>29</v>
       </c>
       <c r="M16" t="str">
-        <v>1666</v>
+        <v>1010</v>
       </c>
       <c r="N16" t="str">
-        <v>396</v>
+        <v>106</v>
       </c>
       <c r="O16" t="str">
-        <v>138</v>
+        <v>28</v>
       </c>
       <c r="P16" t="str">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="Q16" t="str">
         <v>$1,981</v>
@@ -2603,7 +2603,7 @@
         <v>$4,556</v>
       </c>
       <c r="T16" t="str">
-        <v>$3,429</v>
+        <v>$0</v>
       </c>
       <c r="U16" t="str">
         <v>1758</v>
@@ -2725,28 +2725,28 @@
         <v>29</v>
       </c>
       <c r="M17" t="str">
-        <v>656</v>
+        <v>0</v>
       </c>
       <c r="N17" t="str">
-        <v>290</v>
+        <v>0</v>
       </c>
       <c r="O17" t="str">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="P17" t="str">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="str">
-        <v>$1,901</v>
+        <v>$0</v>
       </c>
       <c r="R17" t="str">
-        <v>$2,528</v>
+        <v>$0</v>
       </c>
       <c r="S17" t="str">
-        <v>$4,372</v>
+        <v>$0</v>
       </c>
       <c r="T17" t="str">
-        <v>$3,290</v>
+        <v>$0</v>
       </c>
       <c r="U17" t="str">
         <v>1762</v>
@@ -2868,28 +2868,28 @@
         <v>22</v>
       </c>
       <c r="M18" t="str">
-        <v>1949</v>
+        <v>0</v>
       </c>
       <c r="N18" t="str">
-        <v>236</v>
+        <v>0</v>
       </c>
       <c r="O18" t="str">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="P18" t="str">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="str">
-        <v>$2,609</v>
+        <v>$0</v>
       </c>
       <c r="R18" t="str">
-        <v>$3,470</v>
+        <v>$0</v>
       </c>
       <c r="S18" t="str">
-        <v>$6,001</v>
+        <v>$0</v>
       </c>
       <c r="T18" t="str">
-        <v>$4,519</v>
+        <v>$0</v>
       </c>
       <c r="U18" t="str">
         <v>1949</v>
@@ -3011,16 +3011,16 @@
         <v>25</v>
       </c>
       <c r="M19" t="str">
-        <v>1558</v>
+        <v>846</v>
       </c>
       <c r="N19" t="str">
-        <v>346</v>
+        <v>80</v>
       </c>
       <c r="O19" t="str">
-        <v>118</v>
+        <v>26</v>
       </c>
       <c r="P19" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="Q19" t="str">
         <v>$2,590</v>
@@ -3032,7 +3032,7 @@
         <v>$5,955</v>
       </c>
       <c r="T19" t="str">
-        <v>$4,484</v>
+        <v>$0</v>
       </c>
       <c r="U19" t="str">
         <v>1586</v>
@@ -3127,7 +3127,7 @@
         <v>9,487 km</v>
       </c>
       <c r="D20" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" t="str">
         <v>$15,456</v>
@@ -3136,10 +3136,10 @@
         <v>10</v>
       </c>
       <c r="G20" t="str">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H20" t="str">
-        <v>747-400 (GRU-MXP 2), A380-800 (GRU-0-4)</v>
+        <v>A380-800 (GRU-0-4)</v>
       </c>
       <c r="I20" t="str">
         <v>1957</v>
@@ -3190,13 +3190,13 @@
         <v>27</v>
       </c>
       <c r="Y20" t="str">
-        <v>1957</v>
+        <v>842</v>
       </c>
       <c r="Z20" t="str">
-        <v>340</v>
+        <v>274</v>
       </c>
       <c r="AA20" t="str">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="AB20" t="str">
         <v>27</v>
@@ -3220,7 +3220,7 @@
         <v>MXP</v>
       </c>
       <c r="AI20" t="str">
-        <v>747-400/GRU-MXP 2,A380-800/GRU-0-4</v>
+        <v>A380-800/GRU-0-4</v>
       </c>
       <c r="AJ20">
         <v>1957</v>
@@ -3235,13 +3235,13 @@
         <v>27</v>
       </c>
       <c r="AN20">
-        <v>1957</v>
+        <v>842</v>
       </c>
       <c r="AO20">
-        <v>340</v>
+        <v>274</v>
       </c>
       <c r="AP20">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="AQ20">
         <v>27</v>
@@ -3297,13 +3297,13 @@
         <v>23</v>
       </c>
       <c r="M21" t="str">
-        <v>2506</v>
+        <v>1422</v>
       </c>
       <c r="N21" t="str">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="O21" t="str">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="P21" t="str">
         <v>18</v>
@@ -3440,28 +3440,28 @@
         <v>23</v>
       </c>
       <c r="M22" t="str">
-        <v>1636</v>
+        <v>0</v>
       </c>
       <c r="N22" t="str">
-        <v>232</v>
+        <v>0</v>
       </c>
       <c r="O22" t="str">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="P22" t="str">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q22" t="str">
-        <v>$2,382</v>
+        <v>$0</v>
       </c>
       <c r="R22" t="str">
-        <v>$3,168</v>
+        <v>$0</v>
       </c>
       <c r="S22" t="str">
-        <v>$5,478</v>
+        <v>$0</v>
       </c>
       <c r="T22" t="str">
-        <v>$4,046</v>
+        <v>$0</v>
       </c>
       <c r="U22" t="str">
         <v>1888</v>
@@ -3583,28 +3583,28 @@
         <v>25</v>
       </c>
       <c r="M23" t="str">
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="N23" t="str">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="O23" t="str">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="P23" t="str">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="Q23" t="str">
-        <v>$2,758</v>
+        <v>$0</v>
       </c>
       <c r="R23" t="str">
-        <v>$3,667</v>
+        <v>$0</v>
       </c>
       <c r="S23" t="str">
-        <v>$6,341</v>
+        <v>$0</v>
       </c>
       <c r="T23" t="str">
-        <v>$4,776</v>
+        <v>$0</v>
       </c>
       <c r="U23" t="str">
         <v>1846</v>
@@ -3726,28 +3726,28 @@
         <v>23</v>
       </c>
       <c r="M24" t="str">
-        <v>780</v>
+        <v>0</v>
       </c>
       <c r="N24" t="str">
-        <v>232</v>
+        <v>0</v>
       </c>
       <c r="O24" t="str">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="P24" t="str">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q24" t="str">
-        <v>$2,287</v>
+        <v>$0</v>
       </c>
       <c r="R24" t="str">
-        <v>$3,042</v>
+        <v>$0</v>
       </c>
       <c r="S24" t="str">
-        <v>$5,260</v>
+        <v>$0</v>
       </c>
       <c r="T24" t="str">
-        <v>$3,954</v>
+        <v>$0</v>
       </c>
       <c r="U24" t="str">
         <v>1596</v>
@@ -3842,7 +3842,7 @@
         <v>9,696 km</v>
       </c>
       <c r="D25" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" t="str">
         <v>$12,204</v>
@@ -3851,10 +3851,10 @@
         <v>10</v>
       </c>
       <c r="G25" t="str">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H25" t="str">
-        <v>A350-1000 (GRU-VCE 2), A380-800 (GRU-0-3)</v>
+        <v>A380-800 (GRU-0-3)</v>
       </c>
       <c r="I25" t="str">
         <v>1747</v>
@@ -3869,13 +3869,13 @@
         <v>24</v>
       </c>
       <c r="M25" t="str">
-        <v>1747</v>
+        <v>946</v>
       </c>
       <c r="N25" t="str">
-        <v>303</v>
+        <v>244</v>
       </c>
       <c r="O25" t="str">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="P25" t="str">
         <v>24</v>
@@ -3905,13 +3905,13 @@
         <v>24</v>
       </c>
       <c r="Y25" t="str">
-        <v>1747</v>
+        <v>946</v>
       </c>
       <c r="Z25" t="str">
-        <v>303</v>
+        <v>244</v>
       </c>
       <c r="AA25" t="str">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="AB25" t="str">
         <v>24</v>
@@ -3935,7 +3935,7 @@
         <v>VCE</v>
       </c>
       <c r="AI25" t="str">
-        <v>A350-1000/GRU-VCE 2,A380-800/GRU-0-3</v>
+        <v>A380-800/GRU-0-3</v>
       </c>
       <c r="AJ25">
         <v>1747</v>
@@ -3950,13 +3950,13 @@
         <v>24</v>
       </c>
       <c r="AN25">
-        <v>1747</v>
+        <v>946</v>
       </c>
       <c r="AO25">
-        <v>303</v>
+        <v>244</v>
       </c>
       <c r="AP25">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="AQ25">
         <v>24</v>
@@ -4429,13 +4429,13 @@
         <v>A380-800 (KIX-0-4)</v>
       </c>
       <c r="I29" t="str">
-        <v>1628</v>
+        <v>1677</v>
       </c>
       <c r="J29" t="str">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="K29" t="str">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="L29" t="str">
         <v>27</v>
@@ -4453,25 +4453,25 @@
         <v>27</v>
       </c>
       <c r="Q29" t="str">
-        <v>$2,722</v>
+        <v>$2,612</v>
       </c>
       <c r="R29" t="str">
-        <v>$3,620</v>
+        <v>$3,473</v>
       </c>
       <c r="S29" t="str">
-        <v>$6,260</v>
+        <v>$6,007</v>
       </c>
       <c r="T29" t="str">
-        <v>$4,570</v>
+        <v>$4,571</v>
       </c>
       <c r="U29" t="str">
-        <v>1628</v>
+        <v>1677</v>
       </c>
       <c r="V29" t="str">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="W29" t="str">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="X29" t="str">
         <v>27</v>
@@ -4489,16 +4489,16 @@
         <v>27</v>
       </c>
       <c r="AC29" t="str">
-        <v>$2,722</v>
+        <v>$2,612</v>
       </c>
       <c r="AD29" t="str">
-        <v>$3,620</v>
+        <v>$3,473</v>
       </c>
       <c r="AE29" t="str">
-        <v>$6,260</v>
+        <v>$6,007</v>
       </c>
       <c r="AF29" t="str">
-        <v>$4,570</v>
+        <v>$4,571</v>
       </c>
       <c r="AG29" t="str">
         <v>KIX</v>
@@ -4510,13 +4510,13 @@
         <v>A380-800/KIX-0-4</v>
       </c>
       <c r="AJ29">
-        <v>1628</v>
+        <v>1677</v>
       </c>
       <c r="AK29">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="AL29">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="AM29">
         <v>27</v>
@@ -4534,16 +4534,16 @@
         <v>27</v>
       </c>
       <c r="AR29">
-        <v>2722</v>
+        <v>2612</v>
       </c>
       <c r="AS29">
-        <v>3620</v>
+        <v>3473</v>
       </c>
       <c r="AT29">
-        <v>6260</v>
+        <v>6007</v>
       </c>
       <c r="AU29">
-        <v>4570</v>
+        <v>4571</v>
       </c>
     </row>
     <row r="30">
@@ -4584,28 +4584,28 @@
         <v>22</v>
       </c>
       <c r="M30" t="str">
-        <v>902</v>
+        <v>0</v>
       </c>
       <c r="N30" t="str">
-        <v>172</v>
+        <v>0</v>
       </c>
       <c r="O30" t="str">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="P30" t="str">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="Q30" t="str">
-        <v>$2,506</v>
+        <v>$0</v>
       </c>
       <c r="R30" t="str">
-        <v>$3,332</v>
+        <v>$0</v>
       </c>
       <c r="S30" t="str">
-        <v>$5,763</v>
+        <v>$0</v>
       </c>
       <c r="T30" t="str">
-        <v>$4,448</v>
+        <v>$0</v>
       </c>
       <c r="U30" t="str">
         <v>1878</v>
@@ -5013,28 +5013,28 @@
         <v>28</v>
       </c>
       <c r="M33" t="str">
-        <v>692</v>
+        <v>0</v>
       </c>
       <c r="N33" t="str">
-        <v>278</v>
+        <v>0</v>
       </c>
       <c r="O33" t="str">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="P33" t="str">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="Q33" t="str">
-        <v>$2,052</v>
+        <v>$0</v>
       </c>
       <c r="R33" t="str">
-        <v>$2,660</v>
+        <v>$0</v>
       </c>
       <c r="S33" t="str">
-        <v>$4,424</v>
+        <v>$0</v>
       </c>
       <c r="T33" t="str">
-        <v>$3,642</v>
+        <v>$0</v>
       </c>
       <c r="U33" t="str">
         <v>1696</v>
@@ -5299,28 +5299,28 @@
         <v>21</v>
       </c>
       <c r="M35" t="str">
-        <v>1660</v>
+        <v>0</v>
       </c>
       <c r="N35" t="str">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="O35" t="str">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="P35" t="str">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="str">
-        <v>$2,208</v>
+        <v>$0</v>
       </c>
       <c r="R35" t="str">
-        <v>$2,937</v>
+        <v>$0</v>
       </c>
       <c r="S35" t="str">
-        <v>$5,078</v>
+        <v>$0</v>
       </c>
       <c r="T35" t="str">
-        <v>$3,817</v>
+        <v>$0</v>
       </c>
       <c r="U35" t="str">
         <v>1782</v>
@@ -5585,16 +5585,16 @@
         <v>30</v>
       </c>
       <c r="M37" t="str">
-        <v>1206</v>
+        <v>608</v>
       </c>
       <c r="N37" t="str">
-        <v>356</v>
+        <v>42</v>
       </c>
       <c r="O37" t="str">
-        <v>132</v>
+        <v>4</v>
       </c>
       <c r="P37" t="str">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="str">
         <v>$2,459</v>
@@ -5606,7 +5606,7 @@
         <v>$5,655</v>
       </c>
       <c r="T37" t="str">
-        <v>$4,312</v>
+        <v>$0</v>
       </c>
       <c r="U37" t="str">
         <v>1797</v>
@@ -5871,28 +5871,28 @@
         <v>30</v>
       </c>
       <c r="M39" t="str">
-        <v>720</v>
+        <v>0</v>
       </c>
       <c r="N39" t="str">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="O39" t="str">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P39" t="str">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Q39" t="str">
-        <v>$2,694</v>
+        <v>$0</v>
       </c>
       <c r="R39" t="str">
-        <v>$3,583</v>
+        <v>$0</v>
       </c>
       <c r="S39" t="str">
-        <v>$6,196</v>
+        <v>$0</v>
       </c>
       <c r="T39" t="str">
-        <v>$4,577</v>
+        <v>$0</v>
       </c>
       <c r="U39" t="str">
         <v>1547</v>
@@ -6014,28 +6014,28 @@
         <v>24</v>
       </c>
       <c r="M40" t="str">
-        <v>1730</v>
+        <v>0</v>
       </c>
       <c r="N40" t="str">
-        <v>274</v>
+        <v>0</v>
       </c>
       <c r="O40" t="str">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="P40" t="str">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="Q40" t="str">
-        <v>$2,198</v>
+        <v>$0</v>
       </c>
       <c r="R40" t="str">
-        <v>$2,923</v>
+        <v>$0</v>
       </c>
       <c r="S40" t="str">
-        <v>$5,055</v>
+        <v>$0</v>
       </c>
       <c r="T40" t="str">
-        <v>$3,733</v>
+        <v>$0</v>
       </c>
       <c r="U40" t="str">
         <v>1903</v>
@@ -6157,28 +6157,28 @@
         <v>23</v>
       </c>
       <c r="M41" t="str">
-        <v>776</v>
+        <v>0</v>
       </c>
       <c r="N41" t="str">
-        <v>230</v>
+        <v>0</v>
       </c>
       <c r="O41" t="str">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="P41" t="str">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q41" t="str">
-        <v>$2,191</v>
+        <v>$0</v>
       </c>
       <c r="R41" t="str">
-        <v>$2,848</v>
+        <v>$0</v>
       </c>
       <c r="S41" t="str">
-        <v>$4,753</v>
+        <v>$0</v>
       </c>
       <c r="T41" t="str">
-        <v>$3,888</v>
+        <v>$0</v>
       </c>
       <c r="U41" t="str">
         <v>1457</v>
@@ -6443,28 +6443,28 @@
         <v>27</v>
       </c>
       <c r="M43" t="str">
-        <v>634</v>
+        <v>0</v>
       </c>
       <c r="N43" t="str">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="O43" t="str">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="P43" t="str">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="Q43" t="str">
-        <v>$2,300</v>
+        <v>$0</v>
       </c>
       <c r="R43" t="str">
-        <v>$2,988</v>
+        <v>$0</v>
       </c>
       <c r="S43" t="str">
-        <v>$4,980</v>
+        <v>$0</v>
       </c>
       <c r="T43" t="str">
-        <v>$4,084</v>
+        <v>$0</v>
       </c>
       <c r="U43" t="str">
         <v>1474</v>
@@ -7861,13 +7861,13 @@
         <v>787-9 (LAX-AMS 2), A380-800 (LASV-AMSTERDAM)</v>
       </c>
       <c r="I53" t="str">
-        <v>1536</v>
+        <v>1544</v>
       </c>
       <c r="J53" t="str">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K53" t="str">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="L53" t="str">
         <v>32</v>
@@ -7897,13 +7897,13 @@
         <v>$0</v>
       </c>
       <c r="U53" t="str">
-        <v>1536</v>
+        <v>1544</v>
       </c>
       <c r="V53" t="str">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="W53" t="str">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="X53" t="str">
         <v>32</v>
@@ -7921,16 +7921,16 @@
         <v>32</v>
       </c>
       <c r="AC53" t="str">
-        <v>$2,612</v>
+        <v>$2,570</v>
       </c>
       <c r="AD53" t="str">
-        <v>$3,473</v>
+        <v>$3,418</v>
       </c>
       <c r="AE53" t="str">
-        <v>$6,007</v>
+        <v>$5,910</v>
       </c>
       <c r="AF53" t="str">
-        <v>$4,419</v>
+        <v>$4,411</v>
       </c>
       <c r="AG53" t="str">
         <v>LAX</v>
@@ -7942,13 +7942,13 @@
         <v>787-9/LAX-AMS 2,A380-800/LASV-AMSTERDAM</v>
       </c>
       <c r="AJ53">
-        <v>1536</v>
+        <v>1544</v>
       </c>
       <c r="AK53">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="AL53">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AM53">
         <v>32</v>
@@ -7966,16 +7966,16 @@
         <v>32</v>
       </c>
       <c r="AR53">
-        <v>2612</v>
+        <v>2570</v>
       </c>
       <c r="AS53">
-        <v>3473</v>
+        <v>3418</v>
       </c>
       <c r="AT53">
-        <v>6007</v>
+        <v>5910</v>
       </c>
       <c r="AU53">
-        <v>4419</v>
+        <v>4411</v>
       </c>
     </row>
     <row r="54">
@@ -8159,28 +8159,28 @@
         <v>30</v>
       </c>
       <c r="M55" t="str">
-        <v>578</v>
+        <v>0</v>
       </c>
       <c r="N55" t="str">
-        <v>314</v>
+        <v>0</v>
       </c>
       <c r="O55" t="str">
-        <v>134</v>
+        <v>0</v>
       </c>
       <c r="P55" t="str">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Q55" t="str">
-        <v>$2,741</v>
+        <v>$0</v>
       </c>
       <c r="R55" t="str">
-        <v>$3,645</v>
+        <v>$0</v>
       </c>
       <c r="S55" t="str">
-        <v>$6,303</v>
+        <v>$0</v>
       </c>
       <c r="T55" t="str">
-        <v>$4,748</v>
+        <v>$0</v>
       </c>
       <c r="U55" t="str">
         <v>1406</v>
@@ -8302,25 +8302,25 @@
         <v>30</v>
       </c>
       <c r="M56" t="str">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N56" t="str">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="O56" t="str">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="P56" t="str">
         <v>0</v>
       </c>
       <c r="Q56" t="str">
-        <v>$2,704</v>
+        <v>$0</v>
       </c>
       <c r="R56" t="str">
-        <v>$3,596</v>
+        <v>$0</v>
       </c>
       <c r="S56" t="str">
-        <v>$6,219</v>
+        <v>$0</v>
       </c>
       <c r="T56" t="str">
         <v>$0</v>
@@ -8588,28 +8588,28 @@
         <v>28</v>
       </c>
       <c r="M58" t="str">
-        <v>588</v>
+        <v>0</v>
       </c>
       <c r="N58" t="str">
-        <v>336</v>
+        <v>0</v>
       </c>
       <c r="O58" t="str">
-        <v>122</v>
+        <v>0</v>
       </c>
       <c r="P58" t="str">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="Q58" t="str">
-        <v>$2,658</v>
+        <v>$0</v>
       </c>
       <c r="R58" t="str">
-        <v>$3,535</v>
+        <v>$0</v>
       </c>
       <c r="S58" t="str">
-        <v>$6,113</v>
+        <v>$0</v>
       </c>
       <c r="T58" t="str">
-        <v>$4,564</v>
+        <v>$0</v>
       </c>
       <c r="U58" t="str">
         <v>1707</v>
@@ -8874,25 +8874,25 @@
         <v>29</v>
       </c>
       <c r="M60" t="str">
-        <v>680</v>
+        <v>0</v>
       </c>
       <c r="N60" t="str">
-        <v>192</v>
+        <v>0</v>
       </c>
       <c r="O60" t="str">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="P60" t="str">
         <v>0</v>
       </c>
       <c r="Q60" t="str">
-        <v>$2,589</v>
+        <v>$0</v>
       </c>
       <c r="R60" t="str">
-        <v>$3,443</v>
+        <v>$0</v>
       </c>
       <c r="S60" t="str">
-        <v>$5,954</v>
+        <v>$0</v>
       </c>
       <c r="T60" t="str">
         <v>$0</v>
@@ -9160,28 +9160,28 @@
         <v>20</v>
       </c>
       <c r="M62" t="str">
-        <v>958</v>
+        <v>0</v>
       </c>
       <c r="N62" t="str">
-        <v>228</v>
+        <v>0</v>
       </c>
       <c r="O62" t="str">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="P62" t="str">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="Q62" t="str">
-        <v>$2,731</v>
+        <v>$0</v>
       </c>
       <c r="R62" t="str">
-        <v>$3,632</v>
+        <v>$0</v>
       </c>
       <c r="S62" t="str">
-        <v>$6,281</v>
+        <v>$0</v>
       </c>
       <c r="T62" t="str">
-        <v>$4,689</v>
+        <v>$0</v>
       </c>
       <c r="U62" t="str">
         <v>1243</v>
@@ -9589,25 +9589,25 @@
         <v>27</v>
       </c>
       <c r="M65" t="str">
-        <v>790</v>
+        <v>0</v>
       </c>
       <c r="N65" t="str">
-        <v>224</v>
+        <v>0</v>
       </c>
       <c r="O65" t="str">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="P65" t="str">
         <v>0</v>
       </c>
       <c r="Q65" t="str">
-        <v>$2,585</v>
+        <v>$0</v>
       </c>
       <c r="R65" t="str">
-        <v>$3,438</v>
+        <v>$0</v>
       </c>
       <c r="S65" t="str">
-        <v>$5,945</v>
+        <v>$0</v>
       </c>
       <c r="T65" t="str">
         <v>$0</v>
@@ -9714,10 +9714,10 @@
         <v>10</v>
       </c>
       <c r="G66" t="str">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H66" t="str">
-        <v>A380-800 (LAX-HKG 2), A380-800 (LAX-HKG 1)</v>
+        <v>777-300ER (LAX-0), A380-800 (LAX-HKG 1)</v>
       </c>
       <c r="I66" t="str">
         <v>2088</v>
@@ -9732,28 +9732,28 @@
         <v>32</v>
       </c>
       <c r="M66" t="str">
-        <v>1870</v>
+        <v>0</v>
       </c>
       <c r="N66" t="str">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="O66" t="str">
-        <v>162</v>
+        <v>0</v>
       </c>
       <c r="P66" t="str">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="Q66" t="str">
-        <v>$3,345</v>
+        <v>$0</v>
       </c>
       <c r="R66" t="str">
-        <v>$4,448</v>
+        <v>$0</v>
       </c>
       <c r="S66" t="str">
-        <v>$7,693</v>
+        <v>$0</v>
       </c>
       <c r="T66" t="str">
-        <v>$5,684</v>
+        <v>$0</v>
       </c>
       <c r="U66" t="str">
         <v>2088</v>
@@ -9768,13 +9768,13 @@
         <v>32</v>
       </c>
       <c r="Y66" t="str">
-        <v>1870</v>
+        <v>1666</v>
       </c>
       <c r="Z66" t="str">
-        <v>478</v>
+        <v>348</v>
       </c>
       <c r="AA66" t="str">
-        <v>162</v>
+        <v>122</v>
       </c>
       <c r="AB66" t="str">
         <v>32</v>
@@ -9798,7 +9798,7 @@
         <v>HKG</v>
       </c>
       <c r="AI66" t="str">
-        <v>A380-800/LAX-HKG 2,A380-800/LAX-HKG 1</v>
+        <v>777-300ER/LAX-0,A380-800/LAX-HKG 1</v>
       </c>
       <c r="AJ66">
         <v>2088</v>
@@ -9813,13 +9813,13 @@
         <v>32</v>
       </c>
       <c r="AN66">
-        <v>1870</v>
+        <v>1666</v>
       </c>
       <c r="AO66">
-        <v>478</v>
+        <v>348</v>
       </c>
       <c r="AP66">
-        <v>162</v>
+        <v>122</v>
       </c>
       <c r="AQ66">
         <v>32</v>
@@ -9875,28 +9875,28 @@
         <v>30</v>
       </c>
       <c r="M67" t="str">
-        <v>578</v>
+        <v>0</v>
       </c>
       <c r="N67" t="str">
-        <v>314</v>
+        <v>0</v>
       </c>
       <c r="O67" t="str">
-        <v>134</v>
+        <v>0</v>
       </c>
       <c r="P67" t="str">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Q67" t="str">
-        <v>$2,753</v>
+        <v>$0</v>
       </c>
       <c r="R67" t="str">
-        <v>$3,661</v>
+        <v>$0</v>
       </c>
       <c r="S67" t="str">
-        <v>$6,331</v>
+        <v>$0</v>
       </c>
       <c r="T67" t="str">
-        <v>$4,726</v>
+        <v>$0</v>
       </c>
       <c r="U67" t="str">
         <v>1739</v>
@@ -10018,25 +10018,25 @@
         <v>31</v>
       </c>
       <c r="M68" t="str">
-        <v>1130</v>
+        <v>0</v>
       </c>
       <c r="N68" t="str">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="O68" t="str">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="P68" t="str">
         <v>0</v>
       </c>
       <c r="Q68" t="str">
-        <v>$2,552</v>
+        <v>$0</v>
       </c>
       <c r="R68" t="str">
-        <v>$3,394</v>
+        <v>$0</v>
       </c>
       <c r="S68" t="str">
-        <v>$5,869</v>
+        <v>$0</v>
       </c>
       <c r="T68" t="str">
         <v>$0</v>
@@ -10447,13 +10447,13 @@
         <v>32</v>
       </c>
       <c r="M71" t="str">
-        <v>1422</v>
+        <v>578</v>
       </c>
       <c r="N71" t="str">
-        <v>564</v>
+        <v>314</v>
       </c>
       <c r="O71" t="str">
-        <v>232</v>
+        <v>134</v>
       </c>
       <c r="P71" t="str">
         <v>32</v>
@@ -10590,28 +10590,28 @@
         <v>22</v>
       </c>
       <c r="M72" t="str">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="N72" t="str">
-        <v>270</v>
+        <v>0</v>
       </c>
       <c r="O72" t="str">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P72" t="str">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="Q72" t="str">
-        <v>$2,781</v>
+        <v>$0</v>
       </c>
       <c r="R72" t="str">
-        <v>$3,698</v>
+        <v>$0</v>
       </c>
       <c r="S72" t="str">
-        <v>$6,396</v>
+        <v>$0</v>
       </c>
       <c r="T72" t="str">
-        <v>$4,775</v>
+        <v>$0</v>
       </c>
       <c r="U72" t="str">
         <v>1306</v>
@@ -11019,16 +11019,16 @@
         <v>32</v>
       </c>
       <c r="M75" t="str">
-        <v>1272</v>
+        <v>694</v>
       </c>
       <c r="N75" t="str">
-        <v>398</v>
+        <v>84</v>
       </c>
       <c r="O75" t="str">
-        <v>156</v>
+        <v>22</v>
       </c>
       <c r="P75" t="str">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="Q75" t="str">
         <v>$2,514</v>
@@ -11040,7 +11040,7 @@
         <v>$5,782</v>
       </c>
       <c r="T75" t="str">
-        <v>$4,316</v>
+        <v>$0</v>
       </c>
       <c r="U75" t="str">
         <v>1649</v>
@@ -11162,13 +11162,13 @@
         <v>25</v>
       </c>
       <c r="M76" t="str">
-        <v>1312</v>
+        <v>542</v>
       </c>
       <c r="N76" t="str">
-        <v>364</v>
+        <v>334</v>
       </c>
       <c r="O76" t="str">
-        <v>160</v>
+        <v>134</v>
       </c>
       <c r="P76" t="str">
         <v>25</v>

</xml_diff>

<commit_message>
Otomatik Güncelleme: Uçak ve Rota Excel verileri güncellendi
</commit_message>
<xml_diff>
--- a/routes_output.xlsx
+++ b/routes_output.xlsx
@@ -653,42 +653,42 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>346</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>110</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,768</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,682</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,366</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,795</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -815,42 +815,42 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1396</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>308</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>106</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>24</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,356</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,133</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,418</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,002</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -977,42 +977,42 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1846</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>332</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>104</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>27</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,735</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,637</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,289</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,736</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -1139,42 +1139,42 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>764</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>244</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>76</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>25</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,825</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,757</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,497</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,800</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1301,42 +1301,42 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>952</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>236</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>78</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>23</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,093</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,715</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,516</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,663</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1463,42 +1463,42 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1434</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>254</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>77</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,668</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,548</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,135</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,620</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1625,42 +1625,42 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1582</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>376</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>130</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>27</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,170</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,886</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,991</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,796</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1787,37 +1787,37 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>912</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,234</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,971</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,138</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1949,42 +1949,42 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>566</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>344</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>124</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,197</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,921</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,051</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,803</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -2111,42 +2111,42 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>580</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>340</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>122</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,742</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,646</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,306</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,799</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -2435,44 +2435,44 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q13" t="inlineStr">
         <is>
+          <t>$2,732</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>$3,634</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>$6,284</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
       <c r="U13" t="inlineStr">
         <is>
           <t>1526</t>
@@ -2495,17 +2495,17 @@
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>830</t>
+          <t>1526</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>262</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>79</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -2759,37 +2759,37 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
+          <t>1306</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,704</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,596</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,219</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2921,42 +2921,42 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1666</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>396</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>138</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$1,981</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,635</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,556</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,429</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -3083,42 +3083,42 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>656</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>290</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>110</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$1,901</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,528</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,372</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,290</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -3245,42 +3245,42 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1949</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>236</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>60</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>22</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,609</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,470</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,001</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,519</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -3407,42 +3407,42 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1558</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>346</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>118</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>25</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,590</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,444</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,955</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,484</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -3569,42 +3569,42 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>842</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>274</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>88</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>27</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,662</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,540</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,122</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,659</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -3731,42 +3731,42 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2506</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>124</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>18</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>18</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,633</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,502</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,055</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,560</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -3893,42 +3893,42 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1636</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>232</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>68</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>23</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,382</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,168</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,478</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,046</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -4055,42 +4055,42 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>750</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>250</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>80</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>25</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,758</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,667</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,341</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,776</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -4217,42 +4217,42 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>780</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>232</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>76</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>23</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,287</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,042</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,260</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,954</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -4379,42 +4379,42 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1747</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>303</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>93</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>24</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,718</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,614</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,251</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,758</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -4541,37 +4541,37 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
+          <t>862</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,415</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,212</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,553</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -4865,37 +4865,37 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
+          <t>778</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,723</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,622</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,262</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
@@ -5027,42 +5027,42 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>790</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>284</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>96</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>27</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,706</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,598</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,223</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,580</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -5189,42 +5189,42 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>902</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>172</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>44</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>22</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,506</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,332</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,763</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,448</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -5351,42 +5351,42 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>628</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>312</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>110</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>28</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,483</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,302</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,710</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,353</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -5411,17 +5411,17 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>628</t>
+          <t>1614</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>418</t>
         </is>
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>144</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
@@ -5513,42 +5513,42 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1795</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>321</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>97</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>25</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,598</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,455</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,975</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,396</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -5675,42 +5675,42 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>692</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>278</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>96</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>28</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,052</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,660</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,424</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,642</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -5807,27 +5807,27 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>21</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>A380-800 (KIX-0-3), 767-300ER (KIX-DXB 2)</t>
+          <t>A380-800 (KIX-0-3), 767-300ER (KIX-DXB 2), A350-900ULR (KIX-DXB 2)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2048</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>403</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>131</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -5837,57 +5837,57 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>748</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>298</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>100</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,228</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,963</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,124</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,770</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2048</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>403</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>131</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
@@ -5897,17 +5897,17 @@
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>1372</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>402</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>130</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -5917,22 +5917,22 @@
       </c>
       <c r="AC34" t="inlineStr">
         <is>
-          <t>$2,151</t>
+          <t>$2,228</t>
         </is>
       </c>
       <c r="AD34" t="inlineStr">
         <is>
-          <t>$2,860</t>
+          <t>$2,963</t>
         </is>
       </c>
       <c r="AE34" t="inlineStr">
         <is>
-          <t>$4,947</t>
+          <t>$5,124</t>
         </is>
       </c>
       <c r="AF34" t="inlineStr">
         <is>
-          <t>$3,763</t>
+          <t>$3,770</t>
         </is>
       </c>
     </row>
@@ -5999,42 +5999,42 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1660</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>210</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>56</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,208</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,937</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,078</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,817</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -6323,42 +6323,42 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>356</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>132</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,459</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,270</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,655</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,312</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -6455,22 +6455,22 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>A380-800 (KIX-0-2)</t>
+          <t>777-300ER (KIX-KBP 2), A380-800 (KIX-0-2)</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1917</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>273</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -6485,52 +6485,52 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
+          <t>848</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q38" t="inlineStr">
         <is>
+          <t>$2,355</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>$3,132</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>$5,416</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1917</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>273</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
@@ -6545,42 +6545,42 @@
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1917</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>273</t>
         </is>
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>77</t>
         </is>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>24</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,355</t>
         </is>
       </c>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,132</t>
         </is>
       </c>
       <c r="AE38" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,416</t>
         </is>
       </c>
       <c r="AF38" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,985</t>
         </is>
       </c>
     </row>
@@ -6647,42 +6647,42 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>720</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>250</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>100</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,694</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,583</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,196</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,577</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -6809,42 +6809,42 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1730</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>274</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>77</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>24</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,198</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,923</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,055</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,733</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -6971,42 +6971,42 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1382</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>323</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>107</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>22</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,616</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,479</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,016</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,427</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -7133,42 +7133,42 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>578</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>322</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>114</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>31</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,219</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,881</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,800</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,939</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -7295,42 +7295,42 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1408</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>432</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>160</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>26</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,707</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,600</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,226</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,805</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -7457,42 +7457,42 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1220</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>338</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>120</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,280</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,033</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,244</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,997</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -7943,42 +7943,42 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1806</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>339</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>106</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>26</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,617</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,480</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,019</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,428</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -8105,42 +8105,42 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>578</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>314</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>134</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,444</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,251</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,621</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,286</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -8267,37 +8267,37 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
+          <t>882</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,623</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,488</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,032</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -8429,42 +8429,42 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>808</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>226</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>62</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>27</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,060</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,739</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,738</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,654</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -8591,42 +8591,42 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>648</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>296</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>110</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,206</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,021</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,225</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,859</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -8753,44 +8753,44 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
+          <t>732</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q52" t="inlineStr">
         <is>
+          <t>$2,120</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>$2,819</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>$4,875</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="T52" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
       <c r="U52" t="inlineStr">
         <is>
           <t>2171</t>
@@ -8813,22 +8813,22 @@
       </c>
       <c r="Y52" t="inlineStr">
         <is>
-          <t>732</t>
+          <t>1948</t>
         </is>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>224</t>
         </is>
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>54</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>25</t>
         </is>
       </c>
       <c r="AC52" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="AF52" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,671</t>
         </is>
       </c>
     </row>
@@ -8975,42 +8975,42 @@
       </c>
       <c r="Y53" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1112</t>
         </is>
       </c>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>390</t>
         </is>
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>174</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
       <c r="AC53" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,612</t>
         </is>
       </c>
       <c r="AD53" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,473</t>
         </is>
       </c>
       <c r="AE53" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,007</t>
         </is>
       </c>
       <c r="AF53" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,419</t>
         </is>
       </c>
     </row>
@@ -9077,44 +9077,44 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
+          <t>870</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q54" t="inlineStr">
         <is>
+          <t>$2,571</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>$3,419</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>$5,913</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="S54" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="T54" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
       <c r="U54" t="inlineStr">
         <is>
           <t>1429</t>
@@ -9137,22 +9137,22 @@
       </c>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>870</t>
+          <t>1364</t>
         </is>
       </c>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>480</t>
         </is>
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>189</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="AC54" t="inlineStr">
@@ -9172,7 +9172,7 @@
       </c>
       <c r="AF54" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,367</t>
         </is>
       </c>
     </row>
@@ -9239,42 +9239,42 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>578</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>314</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>134</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,741</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,645</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,303</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,748</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -9401,37 +9401,37 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,704</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,596</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,219</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -9563,42 +9563,42 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>984</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>398</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>162</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,596</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,452</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,970</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,457</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -9725,42 +9725,42 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>588</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>336</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>122</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>28</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,658</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,535</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,113</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,564</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -9887,42 +9887,42 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>578</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>314</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>134</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,610</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,471</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,002</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,480</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -9947,17 +9947,17 @@
       </c>
       <c r="Y59" t="inlineStr">
         <is>
-          <t>578</t>
+          <t>906</t>
         </is>
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>466</t>
         </is>
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>200</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
@@ -10049,37 +10049,37 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
+          <t>680</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>192</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,589</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,443</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,954</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
@@ -10211,42 +10211,42 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>620</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>314</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>114</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,808</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,734</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,458</t>
         </is>
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,820</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -10271,12 +10271,12 @@
       </c>
       <c r="Y61" t="inlineStr">
         <is>
-          <t>620</t>
+          <t>1410</t>
         </is>
       </c>
       <c r="Z61" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>326</t>
         </is>
       </c>
       <c r="AA61" t="inlineStr">
@@ -10373,42 +10373,42 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>958</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>228</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>80</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>20</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,731</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,632</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,281</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,689</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -10535,42 +10535,42 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1296</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>438</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>174</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,669</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,549</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,138</t>
         </is>
       </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,582</t>
         </is>
       </c>
       <c r="U63" t="inlineStr">
@@ -10697,42 +10697,42 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1616</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>352</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>126</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,833</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,767</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,515</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,863</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
@@ -10757,17 +10757,17 @@
       </c>
       <c r="Y64" t="inlineStr">
         <is>
-          <t>608</t>
+          <t>1616</t>
         </is>
       </c>
       <c r="Z64" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>352</t>
         </is>
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>126</t>
         </is>
       </c>
       <c r="AB64" t="inlineStr">
@@ -10859,37 +10859,37 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
+          <t>790</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,585</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,438</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,945</t>
         </is>
       </c>
       <c r="T65" t="inlineStr">
@@ -11021,42 +11021,42 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1870</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>478</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>162</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,345</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,448</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$7,693</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,684</t>
         </is>
       </c>
       <c r="U66" t="inlineStr">
@@ -11081,22 +11081,22 @@
       </c>
       <c r="Y66" t="inlineStr">
         <is>
-          <t>1304</t>
+          <t>1870</t>
         </is>
       </c>
       <c r="Z66" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>478</t>
         </is>
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>162</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
       <c r="AC66" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="AF66" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,684</t>
         </is>
       </c>
     </row>
@@ -11183,42 +11183,42 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>578</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>314</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>134</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,753</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,661</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,331</t>
         </is>
       </c>
       <c r="T67" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,726</t>
         </is>
       </c>
       <c r="U67" t="inlineStr">
@@ -11243,17 +11243,17 @@
       </c>
       <c r="Y67" t="inlineStr">
         <is>
-          <t>578</t>
+          <t>1352</t>
         </is>
       </c>
       <c r="Z67" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>354</t>
         </is>
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>142</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -11345,37 +11345,37 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
+          <t>1130</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P68" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,552</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,394</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,869</t>
         </is>
       </c>
       <c r="T68" t="inlineStr">
@@ -11507,42 +11507,42 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>578</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>314</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>134</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,516</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,346</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,786</t>
         </is>
       </c>
       <c r="T69" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,318</t>
         </is>
       </c>
       <c r="U69" t="inlineStr">
@@ -11567,17 +11567,17 @@
       </c>
       <c r="Y69" t="inlineStr">
         <is>
-          <t>578</t>
+          <t>1096</t>
         </is>
       </c>
       <c r="Z69" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>408</t>
         </is>
       </c>
       <c r="AA69" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>170</t>
         </is>
       </c>
       <c r="AB69" t="inlineStr">
@@ -11669,44 +11669,44 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
+          <t>938</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O70" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P70" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q70" t="inlineStr">
         <is>
+          <t>$2,646</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>$3,519</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>$6,085</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="S70" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="T70" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
       <c r="U70" t="inlineStr">
         <is>
           <t>1490</t>
@@ -11729,22 +11729,22 @@
       </c>
       <c r="Y70" t="inlineStr">
         <is>
-          <t>938</t>
+          <t>1490</t>
         </is>
       </c>
       <c r="Z70" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>442</t>
         </is>
       </c>
       <c r="AA70" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>170</t>
         </is>
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>28</t>
         </is>
       </c>
       <c r="AC70" t="inlineStr">
@@ -11764,7 +11764,7 @@
       </c>
       <c r="AF70" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,495</t>
         </is>
       </c>
     </row>
@@ -11831,42 +11831,42 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1422</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>564</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>232</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,687</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,573</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,180</t>
         </is>
       </c>
       <c r="T71" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,612</t>
         </is>
       </c>
       <c r="U71" t="inlineStr">
@@ -11993,42 +11993,42 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>800</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>100</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>22</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,781</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,698</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,396</t>
         </is>
       </c>
       <c r="T72" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,775</t>
         </is>
       </c>
       <c r="U72" t="inlineStr">
@@ -12155,44 +12155,44 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
+          <t>950</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Q73" t="inlineStr">
         <is>
+          <t>$2,750</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>$3,657</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>$6,324</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="S73" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="T73" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
       <c r="U73" t="inlineStr">
         <is>
           <t>1493</t>
@@ -12215,22 +12215,22 @@
       </c>
       <c r="Y73" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="Z73" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>546</t>
         </is>
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>213</t>
         </is>
       </c>
       <c r="AB73" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>31</t>
         </is>
       </c>
       <c r="AC73" t="inlineStr">
@@ -12250,7 +12250,7 @@
       </c>
       <c r="AF73" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,721</t>
         </is>
       </c>
     </row>
@@ -12317,42 +12317,42 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1262</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>504</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>204</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,801</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,725</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,442</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,759</t>
         </is>
       </c>
       <c r="U74" t="inlineStr">
@@ -12479,42 +12479,42 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1272</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>398</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>156</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,514</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,343</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,782</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,316</t>
         </is>
       </c>
       <c r="U75" t="inlineStr">
@@ -12641,42 +12641,42 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1312</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>364</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>160</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>25</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,581</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,432</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,936</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,431</t>
         </is>
       </c>
       <c r="U76" t="inlineStr">
@@ -12803,42 +12803,42 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1098</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>364</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>154</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,455</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,265</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,445</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,641</t>
         </is>
       </c>
       <c r="U77" t="inlineStr">
@@ -12965,42 +12965,42 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>538</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>340</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>132</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>27</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,578</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,428</t>
         </is>
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$5,929</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,425</t>
         </is>
       </c>
       <c r="U78" t="inlineStr">
@@ -13025,17 +13025,17 @@
       </c>
       <c r="Y78" t="inlineStr">
         <is>
-          <t>538</t>
+          <t>1486</t>
         </is>
       </c>
       <c r="Z78" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>368</t>
         </is>
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>156</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -13127,42 +13127,42 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1376</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>454</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>198</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,815</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,743</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,474</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,833</t>
         </is>
       </c>
       <c r="U79" t="inlineStr">
@@ -13289,42 +13289,42 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1386</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>424</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>156</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>27</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$2,762</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$3,673</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$6,352</t>
         </is>
       </c>
       <c r="T80" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$4,741</t>
         </is>
       </c>
       <c r="U80" t="inlineStr">

</xml_diff>